<commit_message>
updated key_function computation to include ES
</commit_message>
<xml_diff>
--- a/input_processing/key_function_income_thresholds_2018.xlsx
+++ b/input_processing/key_function_income_thresholds_2018.xlsx
@@ -1,20 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/SimPathsEU_AUG/input_processing/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{658B54C1-82E1-ED46-889E-C0905C451111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="results" sheetId="1" r:id="rId2"/>
-    <sheet name="info" sheetId="2" r:id="rId4"/>
+    <sheet name="results" sheetId="1" r:id="rId1"/>
+    <sheet name="info" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="125725" fullCalcOnLoad="true"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="122" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="81">
   <si>
     <t>country</t>
   </si>
@@ -160,9 +167,6 @@
     <t>146 / 315</t>
   </si>
   <si>
-    <t>27484 / .</t>
-  </si>
-  <si>
     <t>181 / 551</t>
   </si>
   <si>
@@ -226,15 +230,9 @@
     <t>Approaches</t>
   </si>
   <si>
-    <t>model_bu = model benefit-unit ID; alternate_bu = plausible raw EUROMOD alternative</t>
-  </si>
-  <si>
     <t>Countries</t>
   </si>
   <si>
-    <t>PL, EL, HU, IT</t>
-  </si>
-  <si>
     <t>Output values</t>
   </si>
   <si>
@@ -245,13 +243,34 @@
   </si>
   <si>
     <t>01_key_function_income_thresholds_from_EUROMOD_2018.do</t>
+  </si>
+  <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>tu_nucfam_HeadID</t>
+  </si>
+  <si>
+    <t>134.83 / 489.33</t>
+  </si>
+  <si>
+    <t>135 / 489</t>
+  </si>
+  <si>
+    <t>model_bu = model benefit-unit ID; alternate_bu = plausible raw EUROMOD alternative (not available for ES)</t>
+  </si>
+  <si>
+    <t>PL, EL, HU, IT, ES</t>
+  </si>
+  <si>
+    <t>27484 / 55312</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -273,29 +292,370 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border/>
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:R10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="11" max="11" width="9.6640625" customWidth="1"/>
+    <col min="12" max="12" width="9.5" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -351,7 +711,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -383,10 +743,10 @@
         <v>30</v>
       </c>
       <c r="K2" s="2">
-        <v>636.23000000000002</v>
+        <v>636.23</v>
       </c>
       <c r="L2" s="2">
-        <v>1360.8900000000001</v>
+        <v>1360.89</v>
       </c>
       <c r="M2" s="2">
         <v>146.31983572895277</v>
@@ -407,7 +767,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -439,7 +799,7 @@
         <v>30</v>
       </c>
       <c r="K3" s="2">
-        <v>636.23000000000002</v>
+        <v>636.23</v>
       </c>
       <c r="L3" s="2">
         <v>1371.5828000000013</v>
@@ -463,24 +823,24 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="E4" s="1">
         <v>2018</v>
       </c>
       <c r="F4" s="1">
-        <v>3568</v>
+        <v>17122</v>
       </c>
       <c r="G4" t="s">
         <v>24</v>
@@ -495,29 +855,31 @@
         <v>30</v>
       </c>
       <c r="K4" s="2">
-        <v>119504.1594</v>
+        <v>586.27859999999998</v>
       </c>
       <c r="L4" s="2">
-        <v>240506.75860000009</v>
+        <v>2127.7215000000006</v>
       </c>
       <c r="M4" s="2">
-        <v>27483.502777823411</v>
+        <v>134.83203942505133</v>
       </c>
       <c r="N4" s="2">
-        <v>55311.615940862444</v>
+        <v>489.33225462012336</v>
       </c>
       <c r="O4" s="1">
-        <v>27484</v>
-      </c>
-      <c r="P4" s="1"/>
+        <v>135</v>
+      </c>
+      <c r="P4" s="1">
+        <v>489</v>
+      </c>
       <c r="Q4" t="s">
-        <v>40</v>
+        <v>76</v>
       </c>
       <c r="R4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -525,10 +887,10 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E5" s="1">
         <v>2018</v>
@@ -563,32 +925,34 @@
       <c r="O5" s="1">
         <v>27484</v>
       </c>
-      <c r="P5" s="1"/>
+      <c r="P5" s="1">
+        <v>55312</v>
+      </c>
       <c r="Q5" t="s">
         <v>40</v>
       </c>
       <c r="R5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E6" s="1">
         <v>2018</v>
       </c>
       <c r="F6" s="1">
-        <v>20544</v>
+        <v>3568</v>
       </c>
       <c r="G6" t="s">
         <v>24</v>
@@ -603,31 +967,31 @@
         <v>30</v>
       </c>
       <c r="K6" s="2">
-        <v>785.7813000000001</v>
+        <v>119504.1594</v>
       </c>
       <c r="L6" s="2">
-        <v>2394.9728999999998</v>
+        <v>240506.75860000009</v>
       </c>
       <c r="M6" s="2">
-        <v>180.71356386036965</v>
+        <v>27483.502777823411</v>
       </c>
       <c r="N6" s="2">
-        <v>550.7945889117043</v>
+        <v>55311.615940862444</v>
       </c>
       <c r="O6" s="1">
-        <v>181</v>
+        <v>27484</v>
       </c>
       <c r="P6" s="1">
-        <v>551</v>
+        <v>55312</v>
       </c>
       <c r="Q6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="R6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -635,16 +999,16 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E7" s="1">
         <v>2018</v>
       </c>
       <c r="F7" s="1">
-        <v>20020</v>
+        <v>20544</v>
       </c>
       <c r="G7" t="s">
         <v>24</v>
@@ -659,48 +1023,48 @@
         <v>30</v>
       </c>
       <c r="K7" s="2">
-        <v>789.10210000000052</v>
+        <v>785.7813000000001</v>
       </c>
       <c r="L7" s="2">
-        <v>2450.3836000000001</v>
+        <v>2394.9728999999998</v>
       </c>
       <c r="M7" s="2">
-        <v>181.47727967145804</v>
+        <v>180.71356386036965</v>
       </c>
       <c r="N7" s="2">
-        <v>563.53791211498981</v>
+        <v>550.7945889117043</v>
       </c>
       <c r="O7" s="1">
         <v>181</v>
       </c>
       <c r="P7" s="1">
-        <v>564</v>
+        <v>551</v>
       </c>
       <c r="Q7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="R7" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E8" s="1">
         <v>2018</v>
       </c>
       <c r="F8" s="1">
-        <v>15484</v>
+        <v>20020</v>
       </c>
       <c r="G8" t="s">
         <v>24</v>
@@ -715,31 +1079,31 @@
         <v>30</v>
       </c>
       <c r="K8" s="2">
-        <v>591.10000000000002</v>
+        <v>789.10210000000052</v>
       </c>
       <c r="L8" s="2">
-        <v>1168.2105000000001</v>
+        <v>2450.3836000000001</v>
       </c>
       <c r="M8" s="2">
-        <v>135.94086242299795</v>
+        <v>181.47727967145804</v>
       </c>
       <c r="N8" s="2">
-        <v>268.66442710472285</v>
+        <v>563.53791211498981</v>
       </c>
       <c r="O8" s="1">
-        <v>136</v>
+        <v>181</v>
       </c>
       <c r="P8" s="1">
-        <v>269</v>
+        <v>564</v>
       </c>
       <c r="Q8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -747,16 +1111,16 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E9" s="1">
         <v>2018</v>
       </c>
       <c r="F9" s="1">
-        <v>14676</v>
+        <v>15484</v>
       </c>
       <c r="G9" t="s">
         <v>24</v>
@@ -771,135 +1135,196 @@
         <v>30</v>
       </c>
       <c r="K9" s="2">
-        <v>606.86000000000001</v>
+        <v>591.1</v>
       </c>
       <c r="L9" s="2">
+        <v>1168.2105000000001</v>
+      </c>
+      <c r="M9" s="2">
+        <v>135.94086242299795</v>
+      </c>
+      <c r="N9" s="2">
+        <v>268.66442710472285</v>
+      </c>
+      <c r="O9" s="1">
+        <v>136</v>
+      </c>
+      <c r="P9" s="1">
+        <v>269</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>43</v>
+      </c>
+      <c r="R9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F10" s="1">
+        <v>14676</v>
+      </c>
+      <c r="G10" t="s">
+        <v>24</v>
+      </c>
+      <c r="H10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J10" t="s">
+        <v>30</v>
+      </c>
+      <c r="K10" s="2">
+        <v>606.86</v>
+      </c>
+      <c r="L10" s="2">
         <v>1247.71</v>
       </c>
-      <c r="M9" s="2">
+      <c r="M10" s="2">
         <v>139.56533880903493</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N10" s="2">
         <v>286.94767967145793</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O10" s="1">
         <v>140</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P10" s="1">
         <v>287</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="Q10" t="s">
         <v>44</v>
       </c>
-      <c r="R9" t="s">
-        <v>52</v>
+      <c r="R10" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="22.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>55</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>57</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>59</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>61</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
         <v>63</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
         <v>65</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
         <v>67</v>
       </c>
-      <c r="B8" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>69</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
+      <c r="B11" t="s">
         <v>71</v>
       </c>
-      <c r="B10" t="s">
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
+      <c r="B12" t="s">
         <v>73</v>
       </c>
-      <c r="B11" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>75</v>
-      </c>
-      <c r="B12" t="s">
-        <v>76</v>
-      </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>